<commit_message>
Fix resigned-employee counting and Physical NTH Salary upload parsing
Count an employee as resigned if either Employment Status says
'Resigned' or a Resigned Date is set, instead of relying on Resigned
Date alone — applied consistently in the Physical dashboard analytics
and HR Analytics V2 overview/circle/CMP breakdowns so both pages agree
on the same headcount.

Also makes the Physical upload's NTH Salary column parsing tolerant of
currency-formatted values (e.g. "₹ 25,000/-") and of header name
casing/spacing variants, so amounts that previously parsed to blank
now save correctly. Physical upload template updated to include the
NTH Salary column.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/formats/physical_format.xlsx
+++ b/frontend/public/formats/physical_format.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECTS FOLDER\SG ENCON\frontend\public\formats\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63097CD8-1954-4524-AAAE-83631F32431B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E849F1E-61A5-4E50-AE25-A2D173F519A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="168">
   <si>
     <t>Cluster</t>
   </si>
@@ -549,6 +549,9 @@
   </si>
   <si>
     <t>Zonal Fiber SME</t>
+  </si>
+  <si>
+    <t>NTH Salary</t>
   </si>
 </sst>
 </file>
@@ -559,7 +562,7 @@
     <numFmt numFmtId="44" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="84">
+  <fonts count="85">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1139,8 +1142,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="42">
+  <fills count="43">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1371,6 +1380,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1726,7 +1741,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="82" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="204" applyFont="1"/>
     <xf numFmtId="9" fontId="74" fillId="0" borderId="0" xfId="204" applyFont="1" applyAlignment="1">
@@ -1737,9 +1752,6 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="204" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="33" borderId="1" xfId="204" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="33" borderId="1" xfId="204" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="34" borderId="11" xfId="204" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="35" borderId="0" xfId="204" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="37" borderId="0" xfId="204" applyFont="1" applyFill="1"/>
@@ -1751,9 +1763,17 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="35" borderId="1" xfId="204" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="39" borderId="1" xfId="204" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="53" fillId="33" borderId="1" xfId="204" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="53" fillId="40" borderId="0" xfId="204" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="41" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="9" fontId="74" fillId="33" borderId="0" xfId="204" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="84" fillId="42" borderId="1" xfId="204" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="42" borderId="1" xfId="204" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="42" borderId="1" xfId="204" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="53" fillId="42" borderId="1" xfId="204" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="205">
     <cellStyle name="20% - Accent1" xfId="41" builtinId="30" customBuiltin="1"/>
@@ -2309,13 +2329,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="18" t="s">
         <v>8</v>
       </c>
       <c r="D1" s="5" t="s">
@@ -2336,7 +2356,7 @@
       <c r="I1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="20" t="s">
         <v>3</v>
       </c>
       <c r="K1" s="5" t="s">
@@ -2360,7 +2380,7 @@
       <c r="Q1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="R1" s="19" t="s">
         <v>13</v>
       </c>
       <c r="S1" s="5" t="s">
@@ -2378,7 +2398,7 @@
       <c r="W1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="X1" s="19" t="s">
         <v>7</v>
       </c>
       <c r="Y1" s="5" t="s">
@@ -2390,7 +2410,7 @@
       <c r="AA1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="AB1" s="16" t="s">
+      <c r="AB1" s="21" t="s">
         <v>126</v>
       </c>
       <c r="AC1" s="5" t="s">
@@ -2405,16 +2425,18 @@
       <c r="AF1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="AG1" s="3"/>
+      <c r="AG1" s="17" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="2" spans="1:33">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="1"/>
@@ -2423,7 +2445,7 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="16" t="s">
         <v>98</v>
       </c>
       <c r="K2" s="1"/>
@@ -2433,7 +2455,7 @@
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
-      <c r="R2" s="9" t="s">
+      <c r="R2" s="8" t="s">
         <v>69</v>
       </c>
       <c r="S2" s="1"/>
@@ -2441,13 +2463,13 @@
       <c r="U2" s="1"/>
       <c r="V2" s="1"/>
       <c r="W2" s="1"/>
-      <c r="X2" s="10" t="s">
+      <c r="X2" s="9" t="s">
         <v>73</v>
       </c>
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
       <c r="AA2" s="1"/>
-      <c r="AB2" s="17" t="s">
+      <c r="AB2" s="15" t="s">
         <v>127</v>
       </c>
       <c r="AC2" s="1"/>
@@ -2457,13 +2479,13 @@
       <c r="AG2" s="3"/>
     </row>
     <row r="3" spans="1:33">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>70</v>
       </c>
       <c r="D3" s="1"/>
@@ -2472,7 +2494,7 @@
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
-      <c r="J3" s="18" t="s">
+      <c r="J3" s="16" t="s">
         <v>95</v>
       </c>
       <c r="K3" s="1"/>
@@ -2482,7 +2504,7 @@
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
-      <c r="R3" s="9" t="s">
+      <c r="R3" s="8" t="s">
         <v>70</v>
       </c>
       <c r="S3" s="1"/>
@@ -2490,13 +2512,13 @@
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
       <c r="W3" s="1"/>
-      <c r="X3" s="10" t="s">
+      <c r="X3" s="9" t="s">
         <v>74</v>
       </c>
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
       <c r="AA3" s="1"/>
-      <c r="AB3" s="17" t="s">
+      <c r="AB3" s="15" t="s">
         <v>71</v>
       </c>
       <c r="AC3" s="1"/>
@@ -2506,13 +2528,13 @@
       <c r="AG3" s="3"/>
     </row>
     <row r="4" spans="1:33">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>71</v>
       </c>
       <c r="D4" s="1"/>
@@ -2521,7 +2543,7 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
-      <c r="J4" s="18" t="s">
+      <c r="J4" s="16" t="s">
         <v>99</v>
       </c>
       <c r="K4" s="1"/>
@@ -2537,13 +2559,13 @@
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
       <c r="W4" s="1"/>
-      <c r="X4" s="10" t="s">
+      <c r="X4" s="9" t="s">
         <v>75</v>
       </c>
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="17" t="s">
+      <c r="AB4" s="15" t="s">
         <v>72</v>
       </c>
       <c r="AC4" s="1"/>
@@ -2553,13 +2575,13 @@
       <c r="AG4" s="3"/>
     </row>
     <row r="5" spans="1:33">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>72</v>
       </c>
       <c r="D5" s="1"/>
@@ -2568,7 +2590,7 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
-      <c r="J5" s="18" t="s">
+      <c r="J5" s="16" t="s">
         <v>100</v>
       </c>
       <c r="K5" s="1"/>
@@ -2596,10 +2618,10 @@
       <c r="AG5" s="3"/>
     </row>
     <row r="6" spans="1:33">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="1"/>
@@ -2609,7 +2631,7 @@
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="18" t="s">
+      <c r="J6" s="16" t="s">
         <v>91</v>
       </c>
       <c r="K6" s="1"/>
@@ -2637,10 +2659,10 @@
       <c r="AG6" s="3"/>
     </row>
     <row r="7" spans="1:33">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>19</v>
       </c>
       <c r="C7" s="1"/>
@@ -2650,7 +2672,7 @@
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
-      <c r="J7" s="18" t="s">
+      <c r="J7" s="16" t="s">
         <v>81</v>
       </c>
       <c r="K7" s="1"/>
@@ -2678,10 +2700,10 @@
       <c r="AG7" s="3"/>
     </row>
     <row r="8" spans="1:33">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C8" s="1"/>
@@ -2691,7 +2713,7 @@
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="18" t="s">
+      <c r="J8" s="16" t="s">
         <v>76</v>
       </c>
       <c r="K8" s="1"/>
@@ -2719,10 +2741,10 @@
       <c r="AG8" s="3"/>
     </row>
     <row r="9" spans="1:33">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C9" s="1"/>
@@ -2732,7 +2754,7 @@
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
-      <c r="J9" s="18" t="s">
+      <c r="J9" s="16" t="s">
         <v>101</v>
       </c>
       <c r="K9" s="1"/>
@@ -2760,10 +2782,10 @@
       <c r="AG9" s="3"/>
     </row>
     <row r="10" spans="1:33">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="1"/>
@@ -2773,7 +2795,7 @@
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
-      <c r="J10" s="18" t="s">
+      <c r="J10" s="16" t="s">
         <v>90</v>
       </c>
       <c r="K10" s="1"/>
@@ -2801,10 +2823,10 @@
       <c r="AG10" s="3"/>
     </row>
     <row r="11" spans="1:33">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>23</v>
       </c>
       <c r="C11" s="1"/>
@@ -2814,7 +2836,7 @@
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="18" t="s">
+      <c r="J11" s="16" t="s">
         <v>88</v>
       </c>
       <c r="K11" s="1"/>
@@ -2851,7 +2873,7 @@
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
-      <c r="J12" s="18" t="s">
+      <c r="J12" s="16" t="s">
         <v>87</v>
       </c>
       <c r="K12" s="1"/>
@@ -2879,211 +2901,211 @@
       <c r="AG12" s="3"/>
     </row>
     <row r="13" spans="1:33">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="J13" s="18" t="s">
+      <c r="J13" s="16" t="s">
         <v>102</v>
       </c>
       <c r="AG13" s="3"/>
     </row>
     <row r="14" spans="1:33">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="J14" s="18" t="s">
+      <c r="J14" s="16" t="s">
         <v>84</v>
       </c>
       <c r="AG14" s="3"/>
     </row>
     <row r="15" spans="1:33">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="J15" s="18" t="s">
+      <c r="J15" s="16" t="s">
         <v>97</v>
       </c>
       <c r="AG15" s="3"/>
     </row>
     <row r="16" spans="1:33">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="J16" s="18" t="s">
+      <c r="J16" s="16" t="s">
         <v>103</v>
       </c>
       <c r="AG16" s="3"/>
     </row>
     <row r="17" spans="1:33">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="J17" s="18" t="s">
+      <c r="J17" s="16" t="s">
         <v>104</v>
       </c>
       <c r="AG17" s="3"/>
     </row>
     <row r="18" spans="1:33">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="J18" s="18" t="s">
+      <c r="J18" s="16" t="s">
         <v>78</v>
       </c>
       <c r="AG18" s="3"/>
     </row>
     <row r="19" spans="1:33">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="J19" s="18" t="s">
+      <c r="J19" s="16" t="s">
         <v>105</v>
       </c>
       <c r="AG19" s="3"/>
     </row>
     <row r="20" spans="1:33">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="J20" s="18" t="s">
+      <c r="J20" s="16" t="s">
         <v>106</v>
       </c>
       <c r="AG20" s="3"/>
     </row>
     <row r="21" spans="1:33">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="J21" s="18" t="s">
+      <c r="J21" s="16" t="s">
         <v>107</v>
       </c>
       <c r="AG21" s="3"/>
     </row>
     <row r="22" spans="1:33">
-      <c r="J22" s="18" t="s">
+      <c r="J22" s="16" t="s">
         <v>79</v>
       </c>
       <c r="AG22" s="3"/>
     </row>
     <row r="23" spans="1:33">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="B23" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="J23" s="18" t="s">
+      <c r="J23" s="16" t="s">
         <v>108</v>
       </c>
       <c r="AG23" s="3"/>
     </row>
     <row r="24" spans="1:33">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B24" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="J24" s="18" t="s">
+      <c r="J24" s="16" t="s">
         <v>109</v>
       </c>
       <c r="AG24" s="3"/>
     </row>
     <row r="25" spans="1:33">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="14" t="s">
+      <c r="B25" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="J25" s="18" t="s">
+      <c r="J25" s="16" t="s">
         <v>86</v>
       </c>
       <c r="AG25" s="3"/>
     </row>
     <row r="26" spans="1:33">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="J26" s="18" t="s">
+      <c r="J26" s="16" t="s">
         <v>82</v>
       </c>
       <c r="AG26" s="3"/>
     </row>
     <row r="27" spans="1:33">
-      <c r="A27" s="14" t="s">
+      <c r="A27" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="14" t="s">
+      <c r="B27" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="J27" s="18" t="s">
+      <c r="J27" s="16" t="s">
         <v>96</v>
       </c>
       <c r="AG27" s="3"/>
     </row>
     <row r="28" spans="1:33">
-      <c r="A28" s="14" t="s">
+      <c r="A28" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="B28" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="J28" s="18" t="s">
+      <c r="J28" s="16" t="s">
         <v>85</v>
       </c>
       <c r="AG28" s="3"/>
     </row>
     <row r="29" spans="1:33">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B29" s="14" t="s">
+      <c r="B29" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="J29" s="18" t="s">
+      <c r="J29" s="16" t="s">
         <v>110</v>
       </c>
       <c r="AG29" s="3"/>
     </row>
     <row r="30" spans="1:33">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="B30" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="J30" s="18" t="s">
+      <c r="J30" s="16" t="s">
         <v>77</v>
       </c>
       <c r="AG30" s="3"/>
@@ -3091,366 +3113,366 @@
     <row r="31" spans="1:33">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
-      <c r="J31" s="18" t="s">
+      <c r="J31" s="16" t="s">
         <v>128</v>
       </c>
       <c r="AG31" s="3"/>
     </row>
     <row r="32" spans="1:33">
-      <c r="A32" s="15" t="s">
+      <c r="A32" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="B32" s="15" t="s">
+      <c r="B32" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="J32" s="18" t="s">
+      <c r="J32" s="16" t="s">
         <v>89</v>
       </c>
       <c r="AG32" s="3"/>
     </row>
     <row r="33" spans="1:33">
-      <c r="A33" s="15" t="s">
+      <c r="A33" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="B33" s="15" t="s">
+      <c r="B33" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="J33" s="18" t="s">
+      <c r="J33" s="16" t="s">
         <v>111</v>
       </c>
       <c r="AG33" s="3"/>
     </row>
     <row r="34" spans="1:33">
-      <c r="A34" s="15" t="s">
+      <c r="A34" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="B34" s="15" t="s">
+      <c r="B34" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="J34" s="18" t="s">
+      <c r="J34" s="16" t="s">
         <v>93</v>
       </c>
       <c r="AG34" s="3"/>
     </row>
     <row r="35" spans="1:33">
-      <c r="A35" s="15" t="s">
+      <c r="A35" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="B35" s="15" t="s">
+      <c r="B35" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="J35" s="18" t="s">
+      <c r="J35" s="16" t="s">
         <v>112</v>
       </c>
       <c r="AG35" s="3"/>
     </row>
     <row r="36" spans="1:33">
-      <c r="A36" s="15" t="s">
+      <c r="A36" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="B36" s="15" t="s">
+      <c r="B36" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="J36" s="18" t="s">
+      <c r="J36" s="16" t="s">
         <v>80</v>
       </c>
       <c r="AG36" s="3"/>
     </row>
     <row r="37" spans="1:33">
-      <c r="A37" s="15" t="s">
+      <c r="A37" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="B37" s="15" t="s">
+      <c r="B37" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="J37" s="18" t="s">
+      <c r="J37" s="16" t="s">
         <v>83</v>
       </c>
       <c r="AG37" s="3"/>
     </row>
     <row r="38" spans="1:33">
-      <c r="A38" s="15" t="s">
+      <c r="A38" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="B38" s="15" t="s">
+      <c r="B38" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="J38" s="18" t="s">
+      <c r="J38" s="16" t="s">
         <v>94</v>
       </c>
       <c r="AG38" s="3"/>
     </row>
     <row r="39" spans="1:33">
-      <c r="J39" s="18" t="s">
+      <c r="J39" s="16" t="s">
         <v>113</v>
       </c>
       <c r="AG39" s="3"/>
     </row>
     <row r="40" spans="1:33">
-      <c r="J40" s="18" t="s">
+      <c r="J40" s="16" t="s">
         <v>114</v>
       </c>
       <c r="AG40" s="3"/>
     </row>
     <row r="41" spans="1:33">
-      <c r="J41" s="18" t="s">
+      <c r="J41" s="16" t="s">
         <v>92</v>
       </c>
       <c r="AG41" s="3"/>
     </row>
     <row r="42" spans="1:33">
-      <c r="J42" s="18" t="s">
+      <c r="J42" s="16" t="s">
         <v>115</v>
       </c>
       <c r="AG42" s="3"/>
     </row>
     <row r="43" spans="1:33">
-      <c r="J43" s="18" t="s">
+      <c r="J43" s="16" t="s">
         <v>116</v>
       </c>
       <c r="AG43" s="3"/>
     </row>
     <row r="44" spans="1:33">
-      <c r="J44" s="18" t="s">
+      <c r="J44" s="16" t="s">
         <v>117</v>
       </c>
       <c r="AG44" s="3"/>
     </row>
     <row r="45" spans="1:33">
-      <c r="J45" s="18" t="s">
+      <c r="J45" s="16" t="s">
         <v>118</v>
       </c>
       <c r="AG45" s="3"/>
     </row>
     <row r="46" spans="1:33">
-      <c r="J46" s="18" t="s">
+      <c r="J46" s="16" t="s">
         <v>119</v>
       </c>
       <c r="AG46" s="3"/>
     </row>
     <row r="47" spans="1:33">
-      <c r="J47" s="18" t="s">
+      <c r="J47" s="16" t="s">
         <v>120</v>
       </c>
       <c r="AG47" s="3"/>
     </row>
     <row r="48" spans="1:33">
-      <c r="J48" s="18" t="s">
+      <c r="J48" s="16" t="s">
         <v>121</v>
       </c>
       <c r="AG48" s="3"/>
     </row>
     <row r="49" spans="10:33">
-      <c r="J49" s="18" t="s">
+      <c r="J49" s="16" t="s">
         <v>122</v>
       </c>
       <c r="AG49" s="3"/>
     </row>
     <row r="50" spans="10:33">
-      <c r="J50" s="18" t="s">
+      <c r="J50" s="16" t="s">
         <v>123</v>
       </c>
       <c r="AG50" s="3"/>
     </row>
     <row r="51" spans="10:33">
-      <c r="J51" s="18" t="s">
+      <c r="J51" s="16" t="s">
         <v>124</v>
       </c>
       <c r="AG51" s="3"/>
     </row>
     <row r="52" spans="10:33">
-      <c r="J52" s="18" t="s">
+      <c r="J52" s="16" t="s">
         <v>125</v>
       </c>
       <c r="AG52" s="3"/>
     </row>
     <row r="53" spans="10:33">
-      <c r="J53" s="18" t="s">
+      <c r="J53" s="16" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="54" spans="10:33">
-      <c r="J54" s="18" t="s">
+      <c r="J54" s="16" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="55" spans="10:33">
-      <c r="J55" s="18" t="s">
+      <c r="J55" s="16" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="56" spans="10:33">
-      <c r="J56" s="18" t="s">
+      <c r="J56" s="16" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="57" spans="10:33">
-      <c r="J57" s="18" t="s">
+      <c r="J57" s="16" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="58" spans="10:33">
-      <c r="J58" s="18" t="s">
+      <c r="J58" s="16" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="59" spans="10:33">
-      <c r="J59" s="18" t="s">
+      <c r="J59" s="16" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="60" spans="10:33">
-      <c r="J60" s="18" t="s">
+      <c r="J60" s="16" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="61" spans="10:33">
-      <c r="J61" s="18" t="s">
+      <c r="J61" s="16" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="62" spans="10:33">
-      <c r="J62" s="18" t="s">
+      <c r="J62" s="16" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="63" spans="10:33">
-      <c r="J63" s="18" t="s">
+      <c r="J63" s="16" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="64" spans="10:33">
-      <c r="J64" s="18" t="s">
+      <c r="J64" s="16" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="65" spans="10:10">
-      <c r="J65" s="18" t="s">
+      <c r="J65" s="16" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="66" spans="10:10">
-      <c r="J66" s="18" t="s">
+      <c r="J66" s="16" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="67" spans="10:10">
-      <c r="J67" s="18" t="s">
+      <c r="J67" s="16" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="68" spans="10:10">
-      <c r="J68" s="18" t="s">
+      <c r="J68" s="16" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="69" spans="10:10">
-      <c r="J69" s="18" t="s">
+      <c r="J69" s="16" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="70" spans="10:10">
-      <c r="J70" s="18" t="s">
+      <c r="J70" s="16" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="71" spans="10:10">
-      <c r="J71" s="18" t="s">
+      <c r="J71" s="16" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="72" spans="10:10">
-      <c r="J72" s="18" t="s">
+      <c r="J72" s="16" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="73" spans="10:10">
-      <c r="J73" s="18" t="s">
+      <c r="J73" s="16" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="74" spans="10:10">
-      <c r="J74" s="18" t="s">
+      <c r="J74" s="16" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="75" spans="10:10">
-      <c r="J75" s="18" t="s">
+      <c r="J75" s="16" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="76" spans="10:10">
-      <c r="J76" s="18" t="s">
+      <c r="J76" s="16" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="77" spans="10:10">
-      <c r="J77" s="18" t="s">
+      <c r="J77" s="16" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="78" spans="10:10">
-      <c r="J78" s="18" t="s">
+      <c r="J78" s="16" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="79" spans="10:10">
-      <c r="J79" s="18" t="s">
+      <c r="J79" s="16" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="80" spans="10:10">
-      <c r="J80" s="18" t="s">
+      <c r="J80" s="16" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="81" spans="10:10">
-      <c r="J81" s="18" t="s">
+      <c r="J81" s="16" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="82" spans="10:10">
-      <c r="J82" s="18" t="s">
+      <c r="J82" s="16" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="83" spans="10:10">
-      <c r="J83" s="18" t="s">
+      <c r="J83" s="16" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="84" spans="10:10">
-      <c r="J84" s="18" t="s">
+      <c r="J84" s="16" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="85" spans="10:10">
-      <c r="J85" s="18" t="s">
+      <c r="J85" s="16" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="86" spans="10:10">
-      <c r="J86" s="18" t="s">
+      <c r="J86" s="16" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="87" spans="10:10">
-      <c r="J87" s="18" t="s">
+      <c r="J87" s="16" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="88" spans="10:10">
-      <c r="J88" s="18" t="s">
+      <c r="J88" s="16" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="89" spans="10:10">
-      <c r="J89" s="18" t="s">
+      <c r="J89" s="16" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="90" spans="10:10">
-      <c r="J90" s="18" t="s">
+      <c r="J90" s="16" t="s">
         <v>166</v>
       </c>
     </row>

</xml_diff>